<commit_message>
Auto update histories + analysis
</commit_message>
<xml_diff>
--- a/data/histories/Anguilla history.xlsx
+++ b/data/histories/Anguilla history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3022"/>
+  <dimension ref="A1:E3023"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82010,6 +82010,33 @@
         </is>
       </c>
     </row>
+    <row r="3023">
+      <c r="A3023" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B3023" t="inlineStr">
+        <is>
+          <t>Anguila 10AM</t>
+        </is>
+      </c>
+      <c r="C3023" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="D3023" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E3023" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>